<commit_message>
docs(task): verify adherence access and report calendar accessibility bug
Refs: 3.24
</commit_message>
<xml_diff>
--- a/work/3.24-adherence-family-view/testcases.xlsx
+++ b/work/3.24-adherence-family-view/testcases.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Family adherence view'!$A$8:$I$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Family adherence view'!$A$8:$I$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -128,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -179,6 +179,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -826,7 +829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1685,10 +1688,14 @@
           <t>200 + audit allowed với A; 403 + audit denied với B/thiếu quyền.</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Backend DB thật: 60 passed; gồm khẳng định tương ứng trong test_adherence_history_access.py.</t>
+        </is>
+      </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -1729,10 +1736,14 @@
           <t>403 ngay request tiếp theo; có audit denied.</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr"/>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Backend DB thật: 60 passed; gồm khẳng định tương ứng trong test_adherence_history_access.py.</t>
+        </is>
+      </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
@@ -1772,10 +1783,14 @@
           <t>Không trả dữ liệu sức khỏe khi audit/quyền lỗi.</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr"/>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Backend DB thật: 60 passed; gồm khẳng định tương ứng trong test_adherence_history_access.py.</t>
+        </is>
+      </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
@@ -1828,61 +1843,109 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
+    <row r="28" ht="74" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-20</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Kiểm vùng chạm chọn ngày ở 320dp</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Flutter test; viewport 320x640; padding ngang 16dp</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>1. Chạy evidence/calendar-accessibility-repro.dart từ frontend/mobile bằng flutter test --no-pub.
+2. Kiểm androidTapTargetGuideline.</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>320dp; ngày 22/10/2026</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Mọi ô tương tác ít nhất 48x48dp.</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>Ô ngày rộng 41.1dp, cao 52dp; androidTapTargetGuideline thất bại.</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>AC9 · BVA viewport 320dp · calendar meets Android tap target sizes at 320dp</t>
+        </is>
+      </c>
+    </row>
     <row r="29"/>
-    <row r="30">
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="H30" s="7">
-        <f>COUNTIF(H9:H27,"Pass")</f>
-        <v/>
-      </c>
-    </row>
+    <row r="30"/>
     <row r="31">
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H31" s="7">
-        <f>COUNTIF(H9:H27,"Fail")</f>
+        <f>COUNTIF(H9:H28,"Pass")</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="H32" s="7">
-        <f>COUNTIF(H9:H27,"Pending")</f>
+        <f>COUNTIF(H9:H28,"Fail")</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="G33" s="6" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H33" s="7">
+        <f>COUNTIF(H9:H28,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="G34" s="6" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="H33" s="7">
-        <f>SUM(H30:H32)</f>
+      <c r="H34" s="7">
+        <f>SUM(H31:H33)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A8:I27"/>
-  <conditionalFormatting sqref="H9:H27">
+  <autoFilter ref="A8:I28"/>
+  <conditionalFormatting sqref="H9:H28">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Fail"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H9:H27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H9:H28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pass,Fail,Pending"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1896,7 +1959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1941,7 +2004,7 @@
         </is>
       </c>
       <c r="C3" s="11">
-        <f>'Family adherence view'!$H$30</f>
+        <f>'Family adherence view'!$H$31</f>
         <v/>
       </c>
       <c r="D3" s="9">
@@ -1957,7 +2020,7 @@
         </is>
       </c>
       <c r="C4" s="11">
-        <f>'Family adherence view'!$H$31</f>
+        <f>'Family adherence view'!$H$32</f>
         <v/>
       </c>
       <c r="D4" s="9">
@@ -1989,7 +2052,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr"/>
       <c r="C6" s="11">
-        <f>'Family adherence view'!$H$32</f>
+        <f>'Family adherence view'!$H$33</f>
         <v/>
       </c>
       <c r="D6" s="9">
@@ -2077,15 +2140,15 @@
         </is>
       </c>
       <c r="D11" s="16">
-        <f>IFERROR(('Family adherence view'!$H$33-'Family adherence view'!$H$32)/'Family adherence view'!$H$33,0)</f>
+        <f>IFERROR(('Family adherence view'!$H$34-'Family adherence view'!$H$33)/'Family adherence view'!$H$34,0)</f>
         <v/>
       </c>
       <c r="E11" s="16">
-        <f>IFERROR('Family adherence view'!$H$30/'Family adherence view'!$H$33,0)</f>
+        <f>IFERROR('Family adherence view'!$H$31/'Family adherence view'!$H$34,0)</f>
         <v/>
       </c>
       <c r="F11" s="16">
-        <f>IFERROR('Family adherence view'!$H$31/'Family adherence view'!$H$33,0)</f>
+        <f>IFERROR('Family adherence view'!$H$32/'Family adherence view'!$H$34,0)</f>
         <v/>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -2095,7 +2158,7 @@
       </c>
       <c r="H11" s="14" t="inlineStr">
         <is>
-          <t>13 Pass tự động; 6 Pending cần thiết bị/DB và kiểm biên đầy đủ.</t>
+          <t>16 Pass, 1 Fail vùng chạm lịch 320dp, 3 Pending manual/biên</t>
         </is>
       </c>
       <c r="I11" s="11" t="inlineStr">
@@ -2155,6 +2218,55 @@
       <c r="I35" s="18" t="inlineStr">
         <is>
           <t>Logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="107" customHeight="1">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>BUG-FAMADH-20</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm vùng chạm chọn ngày ở 320dp</t>
+        </is>
+      </c>
+      <c r="C36" s="19" t="inlineStr">
+        <is>
+          <t>1. Chạy evidence/calendar-accessibility-repro.dart từ frontend/mobile bằng flutter test --no-pub.
+2. Kiểm androidTapTargetGuideline.</t>
+        </is>
+      </c>
+      <c r="D36" s="19" t="inlineStr">
+        <is>
+          <t>320dp; ngày 22/10/2026</t>
+        </is>
+      </c>
+      <c r="E36" s="19" t="inlineStr">
+        <is>
+          <t>Mọi ô tương tác ít nhất 48x48dp.</t>
+        </is>
+      </c>
+      <c r="F36" s="19" t="inlineStr">
+        <is>
+          <t>Ô ngày rộng 41.1dp, cao 52dp; androidTapTargetGuideline thất bại.</t>
+        </is>
+      </c>
+      <c r="G36" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H36" s="19" t="inlineStr">
+        <is>
+          <t>Ngọc Việt</t>
+        </is>
+      </c>
+      <c r="I36" s="19" t="inlineStr">
+        <is>
+          <t>Row chia 7 Expanded vào 288dp còn lại sau padding, mỗi ô chỉ rộng khoảng 41.1dp.
+Log: evidence/test-calendar-accessibility.log</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(task): record passing calendar regression and adherence retest
Refs: 3.24
</commit_message>
<xml_diff>
--- a/work/3.24-adherence-family-view/testcases.xlsx
+++ b/work/3.24-adherence-family-view/testcases.xlsx
@@ -128,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -179,9 +179,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -986,7 +983,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-integration.log.</t>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1033,7 +1030,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-integration.log.</t>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1080,7 +1077,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-integration.log.</t>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1127,7 +1124,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-integration.log.</t>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1174,7 +1171,7 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-integration.log.</t>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1222,7 +1219,7 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-integration.log.</t>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1270,7 +1267,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-integration.log.</t>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -1317,7 +1314,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-integration.log.</t>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1365,7 +1362,7 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-integration.log.</t>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1412,7 +1409,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-integration.log.</t>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1459,7 +1456,7 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-integration.log.</t>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1506,7 +1503,7 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-integration.log.</t>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1553,7 +1550,7 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-integration.log.</t>
+          <t>Khẳng định tự động đạt trong lần chạy Flutter test; xem evidence/test-after-calendar-fix.log.</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1690,7 +1687,7 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Backend DB thật: 60 passed; gồm khẳng định tương ứng trong test_adherence_history_access.py.</t>
+          <t>60 test API/quyền/audit pass trên DB thật sau khi restart Docker, 17.36 giây; khẳng định tương ứng đạt.</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -1738,7 +1735,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Backend DB thật: 60 passed; gồm khẳng định tương ứng trong test_adherence_history_access.py.</t>
+          <t>60 test API/quyền/audit pass trên DB thật sau khi restart Docker, 17.36 giây; khẳng định tương ứng đạt.</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1785,7 +1782,7 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Backend DB thật: 60 passed; gồm khẳng định tương ứng trong test_adherence_history_access.py.</t>
+          <t>60 test API/quyền/audit pass trên DB thật sau khi restart Docker, 17.36 giây; khẳng định tương ứng đạt.</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1831,10 +1828,14 @@
           <t>Chỉ today-89 đến today được chọn; query mỗi lần không quá 90 ngày; tương lai bị khóa.</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr"/>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>Hai ca biên bốn ngày và khóa điều hướng tháng đều pass.</t>
+        </is>
+      </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
@@ -1843,7 +1844,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="74" customHeight="1">
+    <row r="28" ht="90.5" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>TC-FAMADH-20</t>
@@ -1877,17 +1878,17 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Ô ngày rộng 41.1dp, cao 52dp; androidTapTargetGuideline thất bại.</t>
+          <t>Hồi quy tuần/tháng tại 320dp và 375dp, chữ 1.6x đạt androidTapTargetGuideline; chọn ngày cột cuối đúng.</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>AC9 · BVA viewport 320dp · calendar meets Android tap target sizes at 320dp</t>
+          <t>AC9 · BVA viewport 320dp · calendar meets Android tap target sizes at 320dp; BUG-FAMADH-20 đã sửa, giữ log fail cũ test-calendar-accessibility.log</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2158,7 +2159,7 @@
       </c>
       <c r="H11" s="14" t="inlineStr">
         <is>
-          <t>16 Pass, 1 Fail vùng chạm lịch 320dp, 3 Pending manual/biên</t>
+          <t>BUG-FAMADH-20 sửa và pass hồi quy; biên 90 ngày pass; còn manual Figma và thiết bị.</t>
         </is>
       </c>
       <c r="I11" s="11" t="inlineStr">
@@ -2218,55 +2219,6 @@
       <c r="I35" s="18" t="inlineStr">
         <is>
           <t>Logs</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="107" customHeight="1">
-      <c r="A36" s="19" t="inlineStr">
-        <is>
-          <t>BUG-FAMADH-20</t>
-        </is>
-      </c>
-      <c r="B36" s="19" t="inlineStr">
-        <is>
-          <t>Kiểm vùng chạm chọn ngày ở 320dp</t>
-        </is>
-      </c>
-      <c r="C36" s="19" t="inlineStr">
-        <is>
-          <t>1. Chạy evidence/calendar-accessibility-repro.dart từ frontend/mobile bằng flutter test --no-pub.
-2. Kiểm androidTapTargetGuideline.</t>
-        </is>
-      </c>
-      <c r="D36" s="19" t="inlineStr">
-        <is>
-          <t>320dp; ngày 22/10/2026</t>
-        </is>
-      </c>
-      <c r="E36" s="19" t="inlineStr">
-        <is>
-          <t>Mọi ô tương tác ít nhất 48x48dp.</t>
-        </is>
-      </c>
-      <c r="F36" s="19" t="inlineStr">
-        <is>
-          <t>Ô ngày rộng 41.1dp, cao 52dp; androidTapTargetGuideline thất bại.</t>
-        </is>
-      </c>
-      <c r="G36" s="19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H36" s="19" t="inlineStr">
-        <is>
-          <t>Ngọc Việt</t>
-        </is>
-      </c>
-      <c r="I36" s="19" t="inlineStr">
-        <is>
-          <t>Row chia 7 Expanded vào 288dp còn lại sau padding, mỗi ô chỉ rộng khoảng 41.1dp.
-Log: evidence/test-calendar-accessibility.log</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(task): verify master workbook restoration and retain rollover issue
Refs: 3.24
</commit_message>
<xml_diff>
--- a/work/3.24-adherence-family-view/testcases.xlsx
+++ b/work/3.24-adherence-family-view/testcases.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Family adherence view'!$A$8:$I$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Family adherence view'!$A$8:$I$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -128,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -179,6 +179,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -826,7 +829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1892,61 +1895,109 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
+    <row r="29" ht="90.5" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>TC-FAMADH-21</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Giữ khoảng ngày hợp lệ khi refresh qua nửa đêm</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Controller mở ngày 28/10/2026 với selectedDate=31/07/2026 (today-89).</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>1. Chạy evidence/review-date-rollover-repro.dart bằng flutter test --no-pub từ frontend/mobile.
+2. Chuyển đồng hồ sang 29/10/2026 và gọi refresh; xem khoảng request mà repository ghi nhận.</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>now 28/10 → 29/10/2026, selectedDate=31/07/2026</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa ngày đang chọn vào cửa sổ mới trước refresh; mọi request có from&lt;=to.</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Tái hiện request from=01/08/2026, to=31/07/2026. Script tái hiện pass vì khẳng định bug tồn tại; hành vi sản phẩm Fail.</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>AC8 · Chuyển trạng thái đồng hồ · review R2 · có thể chọn ngày khác để tiếp tục</t>
+        </is>
+      </c>
+    </row>
     <row r="30"/>
-    <row r="31">
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="H31" s="7">
-        <f>COUNTIF(H9:H28,"Pass")</f>
-        <v/>
-      </c>
-    </row>
+    <row r="31"/>
     <row r="32">
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="H32" s="7">
-        <f>COUNTIF(H9:H28,"Fail")</f>
+        <f>COUNTIF(H9:H29,"Pass")</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="H33" s="7">
-        <f>COUNTIF(H9:H28,"Pending")</f>
+        <f>COUNTIF(H9:H29,"Fail")</f>
         <v/>
       </c>
     </row>
     <row r="34">
       <c r="G34" s="6" t="inlineStr">
         <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H34" s="7">
+        <f>COUNTIF(H9:H29,"Pending")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="G35" s="6" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="H34" s="7">
-        <f>SUM(H31:H33)</f>
+      <c r="H35" s="7">
+        <f>SUM(H32:H34)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A8:I28"/>
-  <conditionalFormatting sqref="H9:H28">
+  <autoFilter ref="A8:I29"/>
+  <conditionalFormatting sqref="H9:H29">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Fail"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H9:H28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H9:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pass,Fail,Pending"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1960,7 +2011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2005,7 +2056,7 @@
         </is>
       </c>
       <c r="C3" s="11">
-        <f>'Family adherence view'!$H$31</f>
+        <f>'Family adherence view'!$H$32</f>
         <v/>
       </c>
       <c r="D3" s="9">
@@ -2021,7 +2072,7 @@
         </is>
       </c>
       <c r="C4" s="11">
-        <f>'Family adherence view'!$H$32</f>
+        <f>'Family adherence view'!$H$33</f>
         <v/>
       </c>
       <c r="D4" s="9">
@@ -2053,7 +2104,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr"/>
       <c r="C6" s="11">
-        <f>'Family adherence view'!$H$33</f>
+        <f>'Family adherence view'!$H$34</f>
         <v/>
       </c>
       <c r="D6" s="9">
@@ -2141,15 +2192,15 @@
         </is>
       </c>
       <c r="D11" s="16">
-        <f>IFERROR(('Family adherence view'!$H$34-'Family adherence view'!$H$33)/'Family adherence view'!$H$34,0)</f>
+        <f>IFERROR(('Family adherence view'!$H$35-'Family adherence view'!$H$34)/'Family adherence view'!$H$35,0)</f>
         <v/>
       </c>
       <c r="E11" s="16">
-        <f>IFERROR('Family adherence view'!$H$31/'Family adherence view'!$H$34,0)</f>
+        <f>IFERROR('Family adherence view'!$H$32/'Family adherence view'!$H$35,0)</f>
         <v/>
       </c>
       <c r="F11" s="16">
-        <f>IFERROR('Family adherence view'!$H$32/'Family adherence view'!$H$34,0)</f>
+        <f>IFERROR('Family adherence view'!$H$33/'Family adherence view'!$H$35,0)</f>
         <v/>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -2159,7 +2210,7 @@
       </c>
       <c r="H11" s="14" t="inlineStr">
         <is>
-          <t>BUG-FAMADH-20 sửa và pass hồi quy; biên 90 ngày pass; còn manual Figma và thiết bị.</t>
+          <t>R1 workbook đã khôi phục baseline; BUG-FAMADH-20 đã sửa; R2/BUG-FAMADH-21 Medium còn mở; 2 manual Pending.</t>
         </is>
       </c>
       <c r="I11" s="11" t="inlineStr">
@@ -2219,6 +2270,55 @@
       <c r="I35" s="18" t="inlineStr">
         <is>
           <t>Logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="140" customHeight="1">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>BUG-FAMADH-21</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>Giữ khoảng ngày hợp lệ khi refresh qua nửa đêm</t>
+        </is>
+      </c>
+      <c r="C36" s="19" t="inlineStr">
+        <is>
+          <t>1. Chạy evidence/review-date-rollover-repro.dart bằng flutter test --no-pub từ frontend/mobile.
+2. Chuyển đồng hồ sang 29/10/2026 và gọi refresh; xem khoảng request mà repository ghi nhận.</t>
+        </is>
+      </c>
+      <c r="D36" s="19" t="inlineStr">
+        <is>
+          <t>now 28/10 → 29/10/2026, selectedDate=31/07/2026</t>
+        </is>
+      </c>
+      <c r="E36" s="19" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa ngày đang chọn vào cửa sổ mới trước refresh; mọi request có from&lt;=to.</t>
+        </is>
+      </c>
+      <c r="F36" s="19" t="inlineStr">
+        <is>
+          <t>Tái hiện request from=01/08/2026, to=31/07/2026. Script tái hiện pass vì khẳng định bug tồn tại; hành vi sản phẩm Fail.</t>
+        </is>
+      </c>
+      <c r="G36" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H36" s="19" t="inlineStr">
+        <is>
+          <t>Ngọc Việt</t>
+        </is>
+      </c>
+      <c r="I36" s="19" t="inlineStr">
+        <is>
+          <t>selectedDate không được clamp khi earliestDate thay đổi theo đồng hồ; rangeFrom động nhưng rangeTo dựa tháng cũ.
+Log: evidence/test-rollover-known-issue.log</t>
         </is>
       </c>
     </row>

</xml_diff>